<commit_message>
Save work before switching to desktop
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/my-work (outputs)/internal/2026.09.28 - Internal - Cadence Turn-On Tracker.xlsx
+++ b/my-work (outputs)/internal/2026.09.28 - Internal - Cadence Turn-On Tracker.xlsx
@@ -832,7 +832,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Tue 10/13 (Kate approved 10/5). Slips to Tue 10/20 if the Beta Hold suppression is not built in Zoho by Mon 10/12</t>
+          <t>Tue 10/20 (moved from Tue 10/13 on 10/11: Kate sick Thu-Fri, Build RI now Tue 10/13 and Touch 1 Thu 10/15). Slips again if the Ignite Beta Hold suppression isn't built.</t>
         </is>
       </c>
     </row>
@@ -1181,6 +1181,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -1986,7 +1987,7 @@
       <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Due Mon 10/12, or Revenue Intelligence slips to Tue 10/20. Key on email domain, not account name. Spec: Session 3B-ii - GTM Sales/2026.10.05 - Internal - Cadence Build Order and Suppression Check.md</t>
+          <t>Due Mon 10/12, or Revenue Intelligence slips to Tue 10/20. Key on email domain, not account name. Spec: Session 3B-ii - GTM Sales/2026.10.05 - Internal - Cadence Build Order and Suppression Check.md Scheduled Sun 10/11 12:00 to 12:45 CT (Janice, 10/11).</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2010,7 @@
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Runs Mon 10/12 with Touch 2. Target switch-on Tue 10/13.</t>
+          <t>Moved 10/11: runs with RI Touch 2 ahead of the new Tue 10/20 target.</t>
         </is>
       </c>
     </row>

</xml_diff>